<commit_message>
updated the excel cntroller
</commit_message>
<xml_diff>
--- a/uploads/students_template.xlsx
+++ b/uploads/students_template.xlsx
@@ -397,14 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>studentName</v>
       </c>
       <c r="B1" t="str">
-        <v>userName</v>
+        <v>username</v>
       </c>
       <c r="C1" t="str">
         <v>email</v>
@@ -413,25 +413,16 @@
         <v>password</v>
       </c>
       <c r="E1" t="str">
+        <v>phoneNumber</v>
+      </c>
+      <c r="F1" t="str">
         <v>gender</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>birthdate</v>
       </c>
-      <c r="G1" t="str">
-        <v>courseId</v>
-      </c>
       <c r="H1" t="str">
-        <v>courseName</v>
-      </c>
-      <c r="I1" t="str">
-        <v>batchNumber</v>
-      </c>
-      <c r="J1" t="str">
         <v>preferredCourses</v>
-      </c>
-      <c r="K1" t="str">
-        <v>status</v>
       </c>
     </row>
     <row r="2">
@@ -456,19 +447,10 @@
       <c r="G2" t="str">
         <v/>
       </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
student bulk-delete function is added
</commit_message>
<xml_diff>
--- a/uploads/students_template.xlsx
+++ b/uploads/students_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,27 +407,24 @@
         <v>lastName</v>
       </c>
       <c r="C1" t="str">
-        <v>name</v>
+        <v>username</v>
       </c>
       <c r="D1" t="str">
-        <v>username</v>
+        <v>email</v>
       </c>
       <c r="E1" t="str">
-        <v>email</v>
+        <v>password</v>
       </c>
       <c r="F1" t="str">
-        <v>password</v>
+        <v>phoneNumber</v>
       </c>
       <c r="G1" t="str">
-        <v>phoneNumber</v>
+        <v>gender</v>
       </c>
       <c r="H1" t="str">
-        <v>gender</v>
+        <v>birthdate</v>
       </c>
       <c r="I1" t="str">
-        <v>birthdate</v>
-      </c>
-      <c r="J1" t="str">
         <v>preferredCourses</v>
       </c>
     </row>
@@ -456,13 +453,10 @@
       <c r="H2" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>